<commit_message>
Add Azerbaijan (crude) and Israel (crude + refined) to the oil map
- Crude: new hatched-pink Azerbaijan group (Azeri Light, Brent-type) with
  BTC/Ceyhan routes to the EU, Turkey and Israel; Israel added as an
  importer (Azerbaijan 45 / Kazakhstan 25 / Other 30).
- Refined: Israel added as an importer with Russia and USA (JP-8) arrows.
- xlsx sheets and memory.txt kept in sync; all shares sum to 100%.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/OILmap/crude.xlsx
+++ b/OILmap/crude.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -808,6 +808,38 @@
         </is>
       </c>
     </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Pink hatch</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>#e87ba4 (diagonal stripes)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Light, sweet (Azeri Light, ~35–37° API, ~0.15% S)</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Chemically a Brent-type crude (light, sweet, priced off Brent), so hatched in the North Sea pink — linked to but distinct from Norway/UK, same visual treatment as Canada/USA and Kazakhstan/Russia. NOT put with Kazakhstan/Russia: the BTC pipeline (Baku–Tbilisi–Ceyhan) was built to bypass Russia. Placed directly below North Sea in the legend.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -819,7 +851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1962,7 +1994,6 @@
           <t>Round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -1995,7 +2026,6 @@
           <t>Round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr"/>
       <c r="F32" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2028,7 +2058,6 @@
           <t>Across the Atlantic.</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2061,7 +2090,6 @@
           <t>Round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr"/>
       <c r="F34" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2094,7 +2122,6 @@
           <t>Up the Atlantic coast into the US Gulf.</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2127,7 +2154,6 @@
           <t>Dandong–Sinuiju pipeline — North Korea’s main crude supply line.</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2160,7 +2186,6 @@
           <t>Overland / short-haul.</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr"/>
       <c r="F37" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2193,7 +2218,6 @@
           <t>Basrah crude via the Strait of Hormuz.</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2226,7 +2250,6 @@
           <t>Basrah crude via the Strait of Hormuz.</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2259,7 +2282,6 @@
           <t>Via Hormuz and the Strait of Malacca.</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2292,7 +2314,6 @@
           <t>Kirkuk–Ceyhan pipeline.</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2325,7 +2346,6 @@
           <t>Via Hormuz, the Red Sea, Suez and the Atlantic.</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2358,7 +2378,6 @@
           <t>Kazakhstan–China pipeline, overland.</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2391,7 +2410,6 @@
           <t>Short Gulf of Mexico hop; subsidized shipments.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2424,7 +2442,6 @@
           <t>Through the Florida Straits and across the Atlantic.</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr"/>
       <c r="F45" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2457,7 +2474,6 @@
           <t>Across the Atlantic and round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2490,7 +2506,6 @@
           <t>Via the Panama Canal and across the Pacific.</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2523,7 +2538,6 @@
           <t>Across the South Atlantic.</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2556,7 +2570,6 @@
           <t>Across the Atlantic to Eastern Canadian refineries.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2589,7 +2602,6 @@
           <t>Round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2622,7 +2634,6 @@
           <t>Across the Atlantic.</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2655,7 +2666,6 @@
           <t>Short North Sea hop.</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2688,7 +2698,6 @@
           <t>From the Baltic across the Atlantic.</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2721,7 +2730,6 @@
           <t>Druzhba pipeline to Hungary / Slovakia — the last direct Russian crude into the EU.</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2754,7 +2762,6 @@
           <t>Across the Black Sea from Novorossiysk.</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2787,7 +2794,6 @@
           <t>Round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E56" t="inlineStr"/>
       <c r="F56" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2820,7 +2826,6 @@
           <t>Via Suez and across the Atlantic.</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2853,7 +2858,6 @@
           <t>Via the Strait of Hormuz.</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2886,7 +2890,6 @@
           <t>Via the Strait of Hormuz.</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -2919,7 +2922,6 @@
           <t>Via Hormuz and the Strait of Malacca.</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2952,7 +2954,6 @@
           <t>Via Hormuz and the Strait of Malacca.</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr"/>
       <c r="F61" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -2985,7 +2986,6 @@
           <t>Via the Red Sea and Suez.</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr"/>
       <c r="F62" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3018,7 +3018,6 @@
           <t>Via Suez and across the Atlantic.</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3051,7 +3050,6 @@
           <t>The long way round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3084,7 +3082,6 @@
           <t>Across the Atlantic.</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3117,7 +3114,6 @@
           <t>Down the Atlantic coast.</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -3150,7 +3146,6 @@
           <t>Up the East Coast to Eastern Canadian refineries.</t>
         </is>
       </c>
-      <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: always visible</t>
@@ -3183,7 +3178,6 @@
           <t>The long way round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E68" t="inlineStr"/>
       <c r="F68" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3216,7 +3210,6 @@
           <t>Across the Atlantic, mainly to Spain.</t>
         </is>
       </c>
-      <c r="E69" t="inlineStr"/>
       <c r="F69" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
@@ -3249,13 +3242,145 @@
           <t>Across the Atlantic and round the Cape of Good Hope.</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr">
         <is>
           <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
+        <is>
+          <t>~Sept 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>EU</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>~65% of Azerbaijan’s crude exports; ~4.5% of EU crude imports (estimate)</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Baku -&gt; BTC pipeline -&gt; Ceyhan -&gt; Mediterranean tanker -&gt; EU hub (mainly Italy)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>None (pipeline + Mediterranean)</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Project estimate (EU share not in Eurostat headline figures; carved out of "Other suppliers"); map: always visible</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>~Sept 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>~10% of Azerbaijan’s crude exports; ~8% of Turkey’s crude imports</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>BTC pipeline across Georgia into Turkey; feeds SOCAR’s STAR refinery (Aliağa).</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Project estimate (from Export-Import % sheet); map: hidden until selected</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>~Sept 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>~20% of Azerbaijan’s crude exports; ~45% of Israel’s crude imports (~94k bbl/d in 2025)</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Baku -&gt; BTC pipeline -&gt; Ceyhan -&gt; short tanker hop to Haifa/Ashkelon</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Kpler via Jerusalem Post (2025 volume); Oil Change International (Azerbaijan + Kazakhstan ~70%, Nov 2023–Oct 2025); shares estimated; map: always visible</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>~Sept 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>~10% of Kazakhstan’s crude exports; ~25% of Israel’s crude imports</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>CPC pipeline -&gt; Novorossiysk -&gt; Turkish Straits -&gt; Mediterranean</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Oil Change International (combined ~70% with Azerbaijan); split estimated; map: hidden until selected</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
         <is>
           <t>~Sept 2026</t>
         </is>
@@ -3386,7 +3511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -3413,7 +3538,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Brazil and Mexico ARE now tracked (hatched blue "Latin America" group — a regional grouping, not a crude family), and Cuba is tracked as an importer. Still left out: Colombia, Ecuador, Argentina, Guyana (exporters) and Chile/Peru (importers). EU hub import shares are Eurostat-sourced and were NOT changed, so Brazil/Mexico volumes into the EU sit inside its "Other suppliers" 27.8%.</t>
+          <t>Brazil and Mexico ARE now tracked (hatched blue "Latin America" group — a regional grouping, not a crude family), and Cuba is tracked as an importer. Still left out: Colombia, Ecuador, Argentina, Guyana (exporters) and Chile/Peru (importers). EU hub import shares are Eurostat-sourced and were NOT changed, so Brazil/Mexico volumes into the EU sit inside its "Other suppliers" remainder (now 23.3%).</t>
         </is>
       </c>
     </row>
@@ -3462,6 +3587,30 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>On the crude map the US is one point labeled "USA (imports/exports)": it imports more crude than it exports (Canada, Mexico, Venezuela arrows all end there), while its crude export arrows (EU, Asia) still start there. On the refined map the reverse holds — the US is a net exporter of refined products.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Added Sept 2026 as a hatched-pink group (Azeri Light, Brent-type crude). Its EU share (~4.5%) is a project estimate, not Eurostat: it was carved out of the EU "Other suppliers" remainder (27.8% -&gt; 23.3%); every Eurostat-sourced EU share is unchanged. Turkey's "Other" import share dropped 20% -&gt; 12% to make room for Azerbaijan (8%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Added Sept 2026 as an importer (gray). Only Azerbaijan (45%) and Kazakhstan (25%) are drawn; Brazil, Gabon, Nigeria, Angola and others sit in "Other" 30%. To make room: Azerbaijan exports EU 70 -&gt; 65, Other 20 -&gt; 5 (+ Israel 20); Kazakhstan exports Other 15 -&gt; 5 (+ Israel 10).</t>
         </is>
       </c>
     </row>
@@ -3476,7 +3625,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5726,15 +5875,15 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="D90" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>Estimated remainder</t>
+          <t>Estimated; CPC via Novorossiysk and the Turkish Straits</t>
         </is>
       </c>
     </row>
@@ -5746,18 +5895,43 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>Estimated remainder</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
           <t>None</t>
         </is>
       </c>
-      <c r="D91" s="2" t="n">
+      <c r="D92" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="E91" s="2" t="inlineStr">
+      <c r="E92" s="2" t="inlineStr">
         <is>
           <t>Net exporter; no meaningful tracked crude imports</t>
         </is>
@@ -5766,7 +5940,7 @@
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
@@ -5776,32 +5950,32 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="D93" s="2" t="n">
-        <v>0</v>
+        <v>65</v>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>Not tracked as an exporter on this map</t>
+          <t>Estimated; Azeri Light via BTC/Ceyhan, Italy the main buyer</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="D94" s="2" t="n">
@@ -5809,64 +5983,64 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Kpler: ~94k bbl/d to Israel in 2025, ~20% of Azerbaijan’s crude exports</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="D95" s="2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Estimated; BTC pipeline into Turkey (STAR refinery)</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D96" s="2" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Estimated remainder (Israel, Asia and others)</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
@@ -5876,40 +6050,15 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D97" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="B98" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C98" s="2" t="inlineStr">
-        <is>
-          <t>Angola</t>
-        </is>
-      </c>
-      <c r="D98" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="E98" s="2" t="inlineStr">
-        <is>
-          <t>Estimated</t>
+          <t>Net exporter; no meaningful tracked crude imports</t>
         </is>
       </c>
     </row>
@@ -5921,20 +6070,20 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D99" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Not tracked as an exporter on this map</t>
         </is>
       </c>
     </row>
@@ -5951,11 +6100,11 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="D100" s="2" t="n">
-        <v>3</v>
+        <v>20</v>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
@@ -5976,15 +6125,15 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>Brazil</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="D101" s="2" t="n">
-        <v>6</v>
+        <v>15</v>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>Estimated; China is the primary destination for Brazil’s crude</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
@@ -6001,11 +6150,11 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="D102" s="2" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
@@ -6016,32 +6165,32 @@
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="D103" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>Not tracked as an exporter on this map</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -6051,11 +6200,11 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Angola</t>
         </is>
       </c>
       <c r="D104" s="2" t="n">
-        <v>35</v>
+        <v>8</v>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
@@ -6066,7 +6215,7 @@
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -6076,11 +6225,11 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="D105" s="2" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
@@ -6091,7 +6240,7 @@
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
@@ -6101,11 +6250,11 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="D106" s="2" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
@@ -6116,7 +6265,7 @@
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
@@ -6126,22 +6275,22 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="D107" s="2" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Estimated; China is the primary destination for Brazil’s crude</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>China</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
@@ -6151,11 +6300,11 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Nigeria</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D108" s="2" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
@@ -6171,20 +6320,20 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D109" s="2" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Not tracked as an exporter on this map</t>
         </is>
       </c>
     </row>
@@ -6201,11 +6350,11 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="D110" s="2" t="n">
-        <v>12</v>
+        <v>35</v>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
@@ -6216,32 +6365,32 @@
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="D111" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>Not tracked as an exporter on this map</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
@@ -6255,7 +6404,7 @@
         </is>
       </c>
       <c r="D112" s="2" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
@@ -6266,7 +6415,7 @@
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
@@ -6280,7 +6429,7 @@
         </is>
       </c>
       <c r="D113" s="2" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
@@ -6291,7 +6440,7 @@
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
@@ -6301,11 +6450,11 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Nigeria</t>
         </is>
       </c>
       <c r="D114" s="2" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
@@ -6316,7 +6465,7 @@
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>South Korea</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -6326,11 +6475,11 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="D115" s="2" t="n">
-        <v>45</v>
+        <v>4</v>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
@@ -6341,57 +6490,57 @@
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D116" s="2" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Not tracked as an exporter on this map</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D117" s="2" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Not tracked as an exporter on this map</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
@@ -6401,11 +6550,11 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="D118" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
@@ -6416,7 +6565,7 @@
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
@@ -6426,11 +6575,11 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D119" s="2" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
@@ -6441,7 +6590,7 @@
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
@@ -6449,15 +6598,15 @@
           <t>Import</t>
         </is>
       </c>
-      <c r="C120" t="inlineStr">
-        <is>
-          <t>Iran</t>
-        </is>
-      </c>
-      <c r="D120" t="n">
-        <v>5</v>
-      </c>
-      <c r="E120" t="inlineStr">
+      <c r="C120" s="2" t="inlineStr">
+        <is>
+          <t>Iraq</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E120" s="2" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
@@ -6466,7 +6615,7 @@
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>Turkey</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -6480,7 +6629,7 @@
         </is>
       </c>
       <c r="D121" s="2" t="n">
-        <v>20</v>
+        <v>45</v>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
@@ -6491,7 +6640,7 @@
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -6516,7 +6665,7 @@
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -6526,11 +6675,11 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="D123" s="2" t="n">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
@@ -6541,7 +6690,7 @@
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -6551,11 +6700,11 @@
       </c>
       <c r="C124" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="D124" s="2" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
@@ -6566,7 +6715,7 @@
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -6576,11 +6725,11 @@
       </c>
       <c r="C125" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="D125" s="2" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
@@ -6591,132 +6740,132 @@
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Turkey</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C126" s="2" t="inlineStr">
-        <is>
-          <t>EU</t>
-        </is>
-      </c>
-      <c r="D126" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="E126" s="2" t="inlineStr">
-        <is>
-          <t>Estimated; mainly Netherlands and Germany</t>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>5</v>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="127">
-      <c r="A127" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C127" t="inlineStr">
-        <is>
-          <t>China</t>
-        </is>
-      </c>
-      <c r="D127" t="n">
-        <v>15</v>
-      </c>
-      <c r="E127" t="inlineStr">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="B127" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C127" s="2" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E127" s="2" t="inlineStr">
+        <is>
+          <t>Estimated; BTC pipeline, feeds SOCAR’s STAR refinery</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="B128" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C128" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E128" s="2" t="inlineStr">
         <is>
           <t>Estimated</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D128" t="n">
-        <v>10</v>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>Estimated</t>
-        </is>
-      </c>
-    </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>South Korea</t>
-        </is>
-      </c>
-      <c r="D129" t="n">
-        <v>5</v>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>Estimated</t>
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B129" s="2" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C129" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E129" s="2" t="inlineStr">
+        <is>
+          <t>Not an exporter (no domestic crude production)</t>
         </is>
       </c>
     </row>
     <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>United Kingdom</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Export</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D130" t="n">
-        <v>10</v>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>Estimated remainder</t>
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>Israel</t>
+        </is>
+      </c>
+      <c r="B130" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="E130" s="2" t="inlineStr">
+        <is>
+          <t>Kpler 2025 (~46%); Azerbaijan is Israel’s largest crude supplier (BTC/Ceyhan)</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -6726,22 +6875,22 @@
       </c>
       <c r="C131" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="D131" s="2" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Estimated; Oil Change International: Azerbaijan + Kazakhstan ~70%, Nov 2023–Oct 2025</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -6751,72 +6900,72 @@
       </c>
       <c r="C132" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D132" s="2" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Estimated remainder (Brazil, Gabon, Nigeria, Angola, others)</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>United Kingdom</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C133" s="2" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D133" s="2" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>Estimated</t>
+          <t>Not tracked as an exporter on this map</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="C134" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="D134" s="2" t="n">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>Not tracked as an exporter on this map</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
@@ -6826,22 +6975,22 @@
       </c>
       <c r="C135" s="2" t="inlineStr">
         <is>
-          <t>Venezuela</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D135" s="2" t="n">
-        <v>55</v>
+        <v>10</v>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>Estimated; Cuba remains heavily dependent on Venezuelan oil and subsidized shipments for energy and power generation</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -6851,11 +7000,11 @@
       </c>
       <c r="C136" s="2" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D136" s="2" t="n">
-        <v>25</v>
+        <v>55</v>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
@@ -6866,57 +7015,57 @@
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>Cuba</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C137" s="2" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>EU</t>
         </is>
       </c>
       <c r="D137" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="E137" s="2" t="inlineStr">
+        <is>
+          <t>Estimated; mainly Netherlands and Germany</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
         <v>15</v>
       </c>
-      <c r="E137" s="2" t="inlineStr">
+      <c r="E138" t="inlineStr">
         <is>
           <t>Estimated</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" s="2" t="inlineStr">
-        <is>
-          <t>Cuba</t>
-        </is>
-      </c>
-      <c r="B138" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C138" s="2" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D138" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E138" s="2" t="inlineStr">
-        <is>
-          <t>Estimated remainder</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>North Korea</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -6926,122 +7075,122 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Not an exporter</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>North Korea</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>China</t>
+          <t>South Korea</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Estimated; Dandong–Sinuiju pipeline, the main supply line</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>North Korea</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D141" t="n">
+        <v>10</v>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Estimated remainder</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="B142" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C142" s="2" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Estimated; sanctions-busting shipments, rising since 2024</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>North Korea</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Other</t>
-        </is>
-      </c>
-      <c r="D142" t="n">
-        <v>5</v>
-      </c>
-      <c r="E142" t="inlineStr">
-        <is>
-          <t>Estimated remainder</t>
+      <c r="E142" s="2" t="inlineStr">
+        <is>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B143" s="2" t="inlineStr">
         <is>
-          <t>Export</t>
+          <t>Import</t>
         </is>
       </c>
       <c r="C143" s="2" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D143" s="2" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>The EU is drawn as an import hub, not an exporter</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>United Kingdom</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -7051,47 +7200,47 @@
       </c>
       <c r="C144" s="2" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="D144" s="2" t="n">
-        <v>17.8</v>
+        <v>50</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Sourced: Eurostat, Q1 2026</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>Cuba</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>Import</t>
+          <t>Export</t>
         </is>
       </c>
       <c r="C145" s="2" t="inlineStr">
         <is>
-          <t>Norway</t>
+          <t>None</t>
         </is>
       </c>
       <c r="D145" s="2" t="n">
-        <v>16.6</v>
+        <v>0</v>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Sourced: Eurostat, Q1 2026</t>
+          <t>Not tracked as an exporter on this map</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>Cuba</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
@@ -7101,22 +7250,22 @@
       </c>
       <c r="C146" s="2" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Venezuela</t>
         </is>
       </c>
       <c r="D146" s="2" t="n">
-        <v>9.6</v>
+        <v>55</v>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>Sourced: Eurostat, Q1 2026</t>
+          <t>Estimated; Cuba remains heavily dependent on Venezuelan oil and subsidized shipments for energy and power generation</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>Cuba</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
@@ -7126,22 +7275,22 @@
       </c>
       <c r="C147" s="2" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="D147" s="2" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>Sourced: Eurostat, Q1 2026</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>EU (27, hub marker)</t>
+          <t>Cuba</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
@@ -7151,132 +7300,432 @@
       </c>
       <c r="C148" s="2" t="inlineStr">
         <is>
-          <t>Saudi Arabia</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="D148" s="2" t="n">
-        <v>6.8</v>
+        <v>15</v>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>Sourced: Eurostat, Q1 2026</t>
+          <t>Estimated</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
+          <t>Cuba</t>
+        </is>
+      </c>
+      <c r="B149" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C149" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>Estimated remainder</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D150" t="n">
+        <v>0</v>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>Not an exporter</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>China</t>
+        </is>
+      </c>
+      <c r="D151" t="n">
+        <v>65</v>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Estimated; Dandong–Sinuiju pipeline, the main supply line</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="D152" t="n">
+        <v>30</v>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>Estimated; sanctions-busting shipments, rising since 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>North Korea</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>5</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>Estimated remainder</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
           <t>EU (27, hub marker)</t>
         </is>
       </c>
-      <c r="B149" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C149" s="2" t="inlineStr">
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>Export</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>The EU is drawn as an import hub, not an exporter</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>17.8</v>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>Sourced: Eurostat, Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B156" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C156" s="2" t="inlineStr">
+        <is>
+          <t>Norway</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="E156" s="2" t="inlineStr">
+        <is>
+          <t>Sourced: Eurostat, Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B157" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C157" s="2" t="inlineStr">
+        <is>
+          <t>Kazakhstan</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="n">
+        <v>9.6</v>
+      </c>
+      <c r="E157" s="2" t="inlineStr">
+        <is>
+          <t>Sourced: Eurostat, Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B158" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C158" s="2" t="inlineStr">
+        <is>
+          <t>Libya</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E158" s="2" t="inlineStr">
+        <is>
+          <t>Sourced: Eurostat, Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B159" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C159" s="2" t="inlineStr">
+        <is>
+          <t>Saudi Arabia</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="E159" s="2" t="inlineStr">
+        <is>
+          <t>Sourced: Eurostat, Q1 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
         <is>
           <t>Nigeria</t>
         </is>
       </c>
-      <c r="D149" s="2" t="n">
+      <c r="D160" s="2" t="n">
         <v>5.8</v>
       </c>
-      <c r="E149" s="2" t="inlineStr">
+      <c r="E160" s="2" t="inlineStr">
         <is>
           <t>Sourced: Eurostat, Q1 2026</t>
         </is>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" s="2" t="inlineStr">
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
         <is>
           <t>EU (27, hub marker)</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C150" s="2" t="inlineStr">
+      <c r="B161" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C161" s="2" t="inlineStr">
         <is>
           <t>Iraq</t>
         </is>
       </c>
-      <c r="D150" s="2" t="n">
+      <c r="D161" s="2" t="n">
         <v>5.8</v>
       </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="E161" s="2" t="inlineStr">
         <is>
           <t>Sourced: Eurostat, Q1 2026</t>
         </is>
       </c>
     </row>
-    <row r="151">
-      <c r="A151" s="2" t="inlineStr">
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
         <is>
           <t>EU (27, hub marker)</t>
         </is>
       </c>
-      <c r="B151" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C151" s="2" t="inlineStr">
+      <c r="B162" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C162" s="2" t="inlineStr">
+        <is>
+          <t>Azerbaijan</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="E162" s="2" t="inlineStr">
+        <is>
+          <t>Estimated (not in Eurostat headline figures); BTC pipeline via Ceyhan, mainly to Italy</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>EU (27, hub marker)</t>
+        </is>
+      </c>
+      <c r="B163" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C163" s="2" t="inlineStr">
         <is>
           <t>Russia</t>
         </is>
       </c>
-      <c r="D151" s="2" t="n">
+      <c r="D163" s="2" t="n">
         <v>0.8</v>
       </c>
-      <c r="E151" s="2" t="inlineStr">
+      <c r="E163" s="2" t="inlineStr">
         <is>
           <t>Sourced: Eurostat, Q1 2026</t>
         </is>
       </c>
     </row>
-    <row r="152">
-      <c r="A152" s="2" t="inlineStr">
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
         <is>
           <t>EU (27, hub marker)</t>
         </is>
       </c>
-      <c r="B152" s="2" t="inlineStr">
-        <is>
-          <t>Import</t>
-        </is>
-      </c>
-      <c r="C152" s="2" t="inlineStr">
+      <c r="B164" s="2" t="inlineStr">
+        <is>
+          <t>Import</t>
+        </is>
+      </c>
+      <c r="C164" s="2" t="inlineStr">
         <is>
           <t>Other suppliers</t>
         </is>
       </c>
-      <c r="D152" s="2" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="E152" s="2" t="inlineStr">
-        <is>
-          <t>Remainder to reach 100% (unlisted smaller suppliers)</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" s="6" t="inlineStr">
+      <c r="D164" s="2" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="E164" s="2" t="inlineStr">
+        <is>
+          <t>Remainder to reach 100% (unlisted smaller suppliers); Azerbaijan’s estimated 4.5% carved out of it</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="6" t="inlineStr">
         <is>
           <t>EU-27 member states (France, Italy, Spain, Germany, etc.)</t>
         </is>
       </c>
-      <c r="B153" s="6" t="inlineStr">
+      <c r="B165" s="6" t="inlineStr">
         <is>
           <t>Not listed individually. All 27 EU member states hover as one unified "EU" tooltip using the "EU (27, hub marker)" rows above, instead of 27 fragmented entries. Norway and the UK are EU suppliers but not EU members, so they keep separate entries.</t>
         </is>
       </c>
     </row>
-    <row r="154">
-      <c r="A154" s="4" t="inlineStr">
+    <row r="166">
+      <c r="A166" s="4" t="inlineStr">
         <is>
           <t>Note: each country's Export rows sum to 100%, and Import rows sum to 100% (or a single 0% / 'None' row for net exporters with no meaningfully tracked crude imports). Where a hard sourced figure exists it's marked in the notes column; remaining shares are this project's estimates to complete a full 100% picture for the map's hover tooltips — re-verify before treating as authoritative.</t>
         </is>
@@ -7284,7 +7733,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B153:E153"/>
+    <mergeCell ref="B165:E165"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>